<commit_message>
Made ex_trinucleotide_context_metrics.py outpu a per sample JSON
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4AE05A9-ECE0-4438-9905-D12734C63976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{207C6053-CB65-4744-8030-EADFE73496C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="75" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>nn_lower</t>
   </si>
@@ -65,16 +65,28 @@
     <t>Name</t>
   </si>
   <si>
-    <t>placeholder</t>
-  </si>
-  <si>
-    <t>sample</t>
-  </si>
-  <si>
     <t>file_pattern</t>
   </si>
   <si>
     <t>value_pattern</t>
+  </si>
+  <si>
+    <t>ex_trinucleotide_context</t>
+  </si>
+  <si>
+    <t>Comparison of trinucleotide context with established signatures from past studies (cosine similarity score)</t>
+  </si>
+  <si>
+    <t>EX Call somatic variants</t>
+  </si>
+  <si>
+    <t>Sample</t>
+  </si>
+  <si>
+    <t>trinucleotide_context_metrics.txt</t>
+  </si>
+  <si>
+    <t>cosine_similarity_score</t>
   </si>
 </sst>
 </file>
@@ -953,19 +965,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.15625" customWidth="1"/>
-    <col min="2" max="2" width="82.15625" customWidth="1"/>
-    <col min="3" max="4" width="35.26171875" customWidth="1"/>
+    <col min="1" max="1" width="35.140625" customWidth="1"/>
+    <col min="2" max="2" width="82.140625" customWidth="1"/>
+    <col min="3" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.83984375" customWidth="1"/>
-    <col min="10" max="10" width="61.83984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="54" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -994,45 +1006,45 @@
         <v>7</v>
       </c>
       <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="B2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>0.85</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="K2" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added 2 system level metrics to xlsx
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9F887D0-40B7-4431-A644-85E58837123C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49244C7A-8321-44A3-8DD6-15773FB261F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>nn_lower</t>
   </si>
@@ -71,9 +71,6 @@
     <t>value_pattern</t>
   </si>
   <si>
-    <t>ex_trinucleotide_context</t>
-  </si>
-  <si>
     <t>Comparison of trinucleotide context with established signatures from past studies (cosine similarity score)</t>
   </si>
   <si>
@@ -87,6 +84,21 @@
   </si>
   <si>
     <t>EX call somatic variants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of somatic variant calls that are likely to be germline variants </t>
+  </si>
+  <si>
+    <t>Gini coefficient of variant rate between chromosomes</t>
+  </si>
+  <si>
+    <t>chromosomal_variant_rate_uniformity</t>
+  </si>
+  <si>
+    <t>germline_variants_cross_reactivity</t>
+  </si>
+  <si>
+    <t>trinucleotide_context_external_concordance</t>
   </si>
 </sst>
 </file>
@@ -576,10 +588,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="8"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -964,20 +977,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.1796875" customWidth="1"/>
-    <col min="2" max="2" width="82.1796875" customWidth="1"/>
-    <col min="3" max="4" width="35.26953125" customWidth="1"/>
+    <col min="1" max="1" width="41.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="97.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.81640625" customWidth="1"/>
-    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="54" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -1012,18 +1025,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
         <v>12</v>
-      </c>
-      <c r="C2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" t="s">
-        <v>13</v>
       </c>
       <c r="E2">
         <v>0.85</v>
@@ -1041,11 +1054,73 @@
         <v>1</v>
       </c>
       <c r="J2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
         <v>15</v>
       </c>
-      <c r="K2" t="s">
-        <v>14</v>
-      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>3.5</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>1.5</v>
+      </c>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0.2</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0.1</v>
+      </c>
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K82" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>

</xml_diff>

<commit_message>
Started work on chromosomal_variant_rate_metrics.py
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49244C7A-8321-44A3-8DD6-15773FB261F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35CF67C7-3D00-43D9-A1A4-9816BBE8FFD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -71,9 +71,6 @@
     <t>value_pattern</t>
   </si>
   <si>
-    <t>Comparison of trinucleotide context with established signatures from past studies (cosine similarity score)</t>
-  </si>
-  <si>
     <t>Sample</t>
   </si>
   <si>
@@ -86,19 +83,22 @@
     <t>EX call somatic variants</t>
   </si>
   <si>
-    <t xml:space="preserve">Number of somatic variant calls that are likely to be germline variants </t>
-  </si>
-  <si>
-    <t>Gini coefficient of variant rate between chromosomes</t>
-  </si>
-  <si>
-    <t>chromosomal_variant_rate_uniformity</t>
-  </si>
-  <si>
-    <t>germline_variants_cross_reactivity</t>
-  </si>
-  <si>
-    <t>trinucleotide_context_external_concordance</t>
+    <t>ex_trinucleotide_context</t>
+  </si>
+  <si>
+    <t>ex_germline_variants</t>
+  </si>
+  <si>
+    <t>ex_chromosomal_variant_rate_uniformity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percentage of somatic variant calls that are likely to be germline variants </t>
+  </si>
+  <si>
+    <t>Cosine similarity score for trinucleotide context compared with established signatures from past studies</t>
+  </si>
+  <si>
+    <t>Gini coefficient for difference in somatic variant rates between chromosomes</t>
   </si>
 </sst>
 </file>
@@ -1027,16 +1027,16 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
         <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
       </c>
       <c r="E2">
         <v>0.85</v>
@@ -1054,24 +1054,24 @@
         <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1086,23 +1086,23 @@
         <v>1.5</v>
       </c>
       <c r="I3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1117,7 +1117,7 @@
         <v>0.1</v>
       </c>
       <c r="I4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>

</xml_diff>

<commit_message>
Added ex_chromosomal_variant_rate_metrics.py and test
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35CF67C7-3D00-43D9-A1A4-9816BBE8FFD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CAFEEB5-179D-4BC6-B08D-3BE105123BA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
   <si>
     <t>nn_lower</t>
   </si>
@@ -99,6 +99,12 @@
   </si>
   <si>
     <t>Gini coefficient for difference in somatic variant rates between chromosomes</t>
+  </si>
+  <si>
+    <t>_chromosomal_variant_rate_metrics.json</t>
+  </si>
+  <si>
+    <t>gini_coefficient</t>
   </si>
 </sst>
 </file>
@@ -1119,8 +1125,12 @@
       <c r="I4" t="b">
         <v>0</v>
       </c>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
+      <c r="J4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" t="s">
+        <v>22</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K82" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>

</xml_diff>

<commit_message>
Added ex_recurrent_variant_metrics.py and test
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CAFEEB5-179D-4BC6-B08D-3BE105123BA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAAAF344-D3E7-4664-B96C-A6C5CF317094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
   <si>
     <t>nn_lower</t>
   </si>
@@ -86,15 +86,9 @@
     <t>ex_trinucleotide_context</t>
   </si>
   <si>
-    <t>ex_germline_variants</t>
-  </si>
-  <si>
     <t>ex_chromosomal_variant_rate_uniformity</t>
   </si>
   <si>
-    <t xml:space="preserve">Percentage of somatic variant calls that are likely to be germline variants </t>
-  </si>
-  <si>
     <t>Cosine similarity score for trinucleotide context compared with established signatures from past studies</t>
   </si>
   <si>
@@ -105,6 +99,21 @@
   </si>
   <si>
     <t>gini_coefficient</t>
+  </si>
+  <si>
+    <t>ex_unexplained_recurrent_variants</t>
+  </si>
+  <si>
+    <t>Number of somatic variant calls that occur more than once in a batch, without a plausible biological explanation</t>
+  </si>
+  <si>
+    <t>Batch</t>
+  </si>
+  <si>
+    <t>total_recurrent_variants</t>
+  </si>
+  <si>
+    <t>_recurrent_variant_metrics.json</t>
   </si>
 </sst>
 </file>
@@ -594,11 +603,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="8"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -987,7 +995,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="97.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="101.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
@@ -1036,7 +1044,7 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
         <v>14</v>
@@ -1068,41 +1076,45 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C3" t="s">
         <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
       <c r="H3">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I3" t="b">
         <v>0</v>
       </c>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
+      <c r="J3" t="s">
+        <v>25</v>
+      </c>
+      <c r="K3" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
         <v>14</v>
@@ -1123,13 +1135,13 @@
         <v>0.1</v>
       </c>
       <c r="I4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated system level metric names
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F57427D-9555-4947-90FE-EAD9C525C7FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEADB4A1-F394-48FC-B783-6C81A5D3BC98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -86,9 +86,6 @@
     <t>ex_trinucleotide_context</t>
   </si>
   <si>
-    <t>ex_chromosomal_variant_rate_uniformity</t>
-  </si>
-  <si>
     <t>Cosine similarity score for trinucleotide context compared with established signatures from past studies</t>
   </si>
   <si>
@@ -101,9 +98,6 @@
     <t>gini_coefficient</t>
   </si>
   <si>
-    <t>ex_unexplained_recurrent_variants</t>
-  </si>
-  <si>
     <t>Number of somatic variant calls that occur more than once in a batch, without a plausible biological explanation</t>
   </si>
   <si>
@@ -114,6 +108,12 @@
   </si>
   <si>
     <t>_recurrent_variant_metrics.json</t>
+  </si>
+  <si>
+    <t>ex_recurrent_variants</t>
+  </si>
+  <si>
+    <t>ex_chromosomal_variant_rate_gini</t>
   </si>
 </sst>
 </file>
@@ -1044,7 +1044,7 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
         <v>14</v>
@@ -1076,16 +1076,16 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
         <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1103,18 +1103,18 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="K3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
         <v>14</v>
@@ -1138,10 +1138,10 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
+        <v>18</v>
+      </c>
+      <c r="K4" t="s">
         <v>19</v>
-      </c>
-      <c r="K4" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added germline contamination system metric
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEADB4A1-F394-48FC-B783-6C81A5D3BC98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6745EB11-0681-4F56-867B-852973E640C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="30">
   <si>
     <t>nn_lower</t>
   </si>
@@ -114,6 +114,18 @@
   </si>
   <si>
     <t>ex_chromosomal_variant_rate_gini</t>
+  </si>
+  <si>
+    <t>ex_germline_contamination</t>
+  </si>
+  <si>
+    <t>Percentage of somatic variants that are germline contaminants</t>
+  </si>
+  <si>
+    <t>_germline_matches.json</t>
+  </si>
+  <si>
+    <t>percent_germline_contamination</t>
   </si>
 </sst>
 </file>
@@ -991,7 +1003,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.85546875" bestFit="1" customWidth="1"/>
@@ -1144,6 +1156,41 @@
         <v>19</v>
       </c>
     </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K5" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K82" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
1. Added implicit parameters to config 2. Added metrics files for ms_remove_duplicates
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6745EB11-0681-4F56-867B-852973E640C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B25090CE-DC48-4F4E-8975-812898EB99F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -122,10 +122,10 @@
     <t>Percentage of somatic variants that are germline contaminants</t>
   </si>
   <si>
-    <t>_germline_matches.json</t>
-  </si>
-  <si>
     <t>percent_germline_contamination</t>
+  </si>
+  <si>
+    <t>_germline_contamination_metrics.json</t>
   </si>
 </sst>
 </file>
@@ -1185,10 +1185,10 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K5" t="s">
         <v>28</v>
-      </c>
-      <c r="K5" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated trinucleotide context scripts to compare to multiple contexts
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B25090CE-DC48-4F4E-8975-812898EB99F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C979A822-2152-4A26-A2C5-9800A6A0B767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -1004,19 +1004,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
   <dimension ref="A1:K5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="41.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="101.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="35.28515625" customWidth="1"/>
+    <col min="1" max="1" width="41.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="101.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="35.26953125" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" customWidth="1"/>
-    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.81640625" customWidth="1"/>
+    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="54" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -1051,7 +1051,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -1077,7 +1077,7 @@
         <v>1</v>
       </c>
       <c r="I2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
@@ -1086,7 +1086,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -1121,7 +1121,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -1156,7 +1156,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>26</v>
       </c>

</xml_diff>

<commit_message>
Added back trinucleotide context to metrics report
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C979A822-2152-4A26-A2C5-9800A6A0B767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFE3A641-0075-4B76-82AA-A4D9E24416AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -74,12 +74,6 @@
     <t>Sample</t>
   </si>
   <si>
-    <t>cosine_similarity_score</t>
-  </si>
-  <si>
-    <t>_trinucleotide_context_metrics.json</t>
-  </si>
-  <si>
     <t>EX call somatic variants</t>
   </si>
   <si>
@@ -126,6 +120,12 @@
   </si>
   <si>
     <t>_germline_contamination_metrics.json</t>
+  </si>
+  <si>
+    <t>_trinuc_similarities.csv</t>
+  </si>
+  <si>
+    <t>^Abascal-2021-granulocyte,(?P&lt;val&gt;[0-9.]+)$</t>
   </si>
 </sst>
 </file>
@@ -1053,13 +1053,13 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
         <v>11</v>
@@ -1077,27 +1077,27 @@
         <v>1</v>
       </c>
       <c r="I2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="K2" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1115,21 +1115,21 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
@@ -1150,21 +1150,21 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="K4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
@@ -1185,10 +1185,10 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New metric that calculates distance to nearest SNV, and calculates percentiles. Added component metric relating to this
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFE3A641-0075-4B76-82AA-A4D9E24416AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99463EDA-8154-446C-AE82-E8E771A446B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$83</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
   <si>
     <t>nn_lower</t>
   </si>
@@ -126,6 +126,18 @@
   </si>
   <si>
     <t>^Abascal-2021-granulocyte,(?P&lt;val&gt;[0-9.]+)$</t>
+  </si>
+  <si>
+    <t>ex_snv_distance</t>
+  </si>
+  <si>
+    <t>5th percentile of distance of each SNV to nearest SNV</t>
+  </si>
+  <si>
+    <t>_snv_distance.json</t>
+  </si>
+  <si>
+    <t>percentiles.5</t>
   </si>
 </sst>
 </file>
@@ -1003,7 +1015,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="41.81640625" bestFit="1" customWidth="1"/>
@@ -1088,80 +1100,80 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>3000000</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>1500000</v>
       </c>
       <c r="I3" t="b">
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="K3" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="G4">
         <v>0</v>
       </c>
       <c r="H4">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="I4" t="b">
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="K4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
@@ -1173,26 +1185,61 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I5" t="b">
         <v>1</v>
       </c>
       <c r="J5" t="s">
+        <v>16</v>
+      </c>
+      <c r="K5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6" t="s">
         <v>27</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K6" t="s">
         <v>26</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K82" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K83" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Added system metric to assess SNV position vs uniform distribution
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99463EDA-8154-446C-AE82-E8E771A446B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50D3FDBB-7351-410C-9ECD-A0E6F5D874C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
   <si>
     <t>nn_lower</t>
   </si>
@@ -138,6 +138,18 @@
   </si>
   <si>
     <t>percentiles.5</t>
+  </si>
+  <si>
+    <t>ex_snv_position</t>
+  </si>
+  <si>
+    <t>Mean absolute deviation between SNV distribution and uniform distribution for each chrom. Highest chrom compared to target.</t>
+  </si>
+  <si>
+    <t>_snv_position_metrics.json</t>
+  </si>
+  <si>
+    <t>max_MAD</t>
   </si>
 </sst>
 </file>
@@ -1015,7 +1027,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="41.81640625" bestFit="1" customWidth="1"/>
@@ -1065,10 +1077,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -1077,25 +1089,25 @@
         <v>11</v>
       </c>
       <c r="E2">
-        <v>0.85</v>
+        <v>0</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G2">
-        <v>0.95</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I2" t="b">
         <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="K2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
@@ -1135,72 +1147,72 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="G4">
         <v>0</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I4" t="b">
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="K4" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="I5" t="b">
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="K5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
@@ -1236,6 +1248,41 @@
       </c>
       <c r="K6" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7">
+        <v>0.85</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>0.95</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" t="s">
+        <v>28</v>
+      </c>
+      <c r="K7" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated system metric thresholds
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50D3FDBB-7351-410C-9ECD-A0E6F5D874C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC966B2F-354A-4706-A895-DF9C30295949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -1232,13 +1232,13 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I6" t="b">
         <v>1</v>
@@ -1264,7 +1264,7 @@
         <v>11</v>
       </c>
       <c r="E7">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="F7">
         <v>1</v>

</xml_diff>

<commit_message>
ex_snv_position now uses average MAD rather than max MAD
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC966B2F-354A-4706-A895-DF9C30295949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{587127F4-6A24-4276-976B-796B4E4571DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -143,13 +143,13 @@
     <t>ex_snv_position</t>
   </si>
   <si>
-    <t>Mean absolute deviation between SNV distribution and uniform distribution for each chrom. Highest chrom compared to target.</t>
-  </si>
-  <si>
     <t>_snv_position_metrics.json</t>
   </si>
   <si>
-    <t>max_MAD</t>
+    <t>Mean absolute deviation between SNV distribution and uniform distribution for each chrom. Average for all chroms compared to target.</t>
+  </si>
+  <si>
+    <t>mean_MAD</t>
   </si>
 </sst>
 </file>
@@ -1080,7 +1080,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -1104,7 +1104,7 @@
         <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K2" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Added System Level metrics that are not assessed bioinformatically
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{587127F4-6A24-4276-976B-796B4E4571DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDBA57B8-9805-40E8-9B94-346929B83360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="50">
   <si>
     <t>nn_lower</t>
   </si>
@@ -77,9 +77,6 @@
     <t>EX call somatic variants</t>
   </si>
   <si>
-    <t>ex_trinucleotide_context</t>
-  </si>
-  <si>
     <t>Cosine similarity score for trinucleotide context compared with established signatures from past studies</t>
   </si>
   <si>
@@ -104,15 +101,6 @@
     <t>_recurrent_variant_metrics.json</t>
   </si>
   <si>
-    <t>ex_recurrent_variants</t>
-  </si>
-  <si>
-    <t>ex_chromosomal_variant_rate_gini</t>
-  </si>
-  <si>
-    <t>ex_germline_contamination</t>
-  </si>
-  <si>
     <t>Percentage of somatic variants that are germline contaminants</t>
   </si>
   <si>
@@ -128,9 +116,6 @@
     <t>^Abascal-2021-granulocyte,(?P&lt;val&gt;[0-9.]+)$</t>
   </si>
   <si>
-    <t>ex_snv_distance</t>
-  </si>
-  <si>
     <t>5th percentile of distance of each SNV to nearest SNV</t>
   </si>
   <si>
@@ -140,9 +125,6 @@
     <t>percentiles.5</t>
   </si>
   <si>
-    <t>ex_snv_position</t>
-  </si>
-  <si>
     <t>_snv_position_metrics.json</t>
   </si>
   <si>
@@ -150,6 +132,60 @@
   </si>
   <si>
     <t>mean_MAD</t>
+  </si>
+  <si>
+    <t>Precision (inter batch)</t>
+  </si>
+  <si>
+    <t>Precision (intra batch)</t>
+  </si>
+  <si>
+    <t>Linearity</t>
+  </si>
+  <si>
+    <t>Coefficient of variation of technical replicates (%CV)</t>
+  </si>
+  <si>
+    <t>Correlation between two batches, each sample run in both batches (Pearson's R)</t>
+  </si>
+  <si>
+    <t>Linearity of response of varying ratios of blood (high mutation) and sperm (low mutation) from the same donor (R^2)</t>
+  </si>
+  <si>
+    <t>External concodance (blood)</t>
+  </si>
+  <si>
+    <t>External concordance (sperm)</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Number of SNVs per diploid genome is similar to past studies (mean)</t>
+  </si>
+  <si>
+    <t>Robustness</t>
+  </si>
+  <si>
+    <t>Percentage of samples that meet all non-negotiable metrics (including samples which failed processing)</t>
+  </si>
+  <si>
+    <t>Uniformity (SNV position)</t>
+  </si>
+  <si>
+    <t>Uniformity (SNV spacing)</t>
+  </si>
+  <si>
+    <t>Uniformity (chromosomal SNV rate)</t>
+  </si>
+  <si>
+    <t>Cross-reactivity (recurrent variants)</t>
+  </si>
+  <si>
+    <t>External concordance (trinucleotide context)</t>
+  </si>
+  <si>
+    <t>Cross-reactivity (germline contamination)</t>
   </si>
 </sst>
 </file>
@@ -639,10 +675,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1027,7 +1062,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="41.81640625" bestFit="1" customWidth="1"/>
@@ -1068,7 +1103,7 @@
       <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
@@ -1077,10 +1112,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -1104,18 +1139,18 @@
         <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="K2" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
@@ -1139,18 +1174,18 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="K3" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
         <v>12</v>
@@ -1174,24 +1209,24 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
+        <v>15</v>
+      </c>
+      <c r="K4" t="s">
         <v>16</v>
-      </c>
-      <c r="K4" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1209,18 +1244,18 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
         <v>12</v>
@@ -1244,18 +1279,18 @@
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="K6" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" t="s">
         <v>13</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
@@ -1279,10 +1314,220 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="K7" t="s">
-        <v>29</v>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>400</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>200</v>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
+      <c r="J8" t="s">
+        <v>40</v>
+      </c>
+      <c r="K8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9">
+        <v>500</v>
+      </c>
+      <c r="F9">
+        <v>5000</v>
+      </c>
+      <c r="G9">
+        <v>1000</v>
+      </c>
+      <c r="H9">
+        <v>2500</v>
+      </c>
+      <c r="I9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J9" t="s">
+        <v>40</v>
+      </c>
+      <c r="K9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>20</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>10</v>
+      </c>
+      <c r="I10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J10" t="s">
+        <v>40</v>
+      </c>
+      <c r="K10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11">
+        <v>0.9</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>0.95</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11" t="b">
+        <v>0</v>
+      </c>
+      <c r="J11" t="s">
+        <v>40</v>
+      </c>
+      <c r="K11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12">
+        <v>0.9</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>0.95</v>
+      </c>
+      <c r="H12">
+        <v>1</v>
+      </c>
+      <c r="I12" t="b">
+        <v>0</v>
+      </c>
+      <c r="J12" t="s">
+        <v>40</v>
+      </c>
+      <c r="K12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13">
+        <v>90</v>
+      </c>
+      <c r="F13">
+        <v>100</v>
+      </c>
+      <c r="G13">
+        <v>95</v>
+      </c>
+      <c r="H13">
+        <v>100</v>
+      </c>
+      <c r="I13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J13" t="s">
+        <v>40</v>
+      </c>
+      <c r="K13" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed system metrics regex bug
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDBA57B8-9805-40E8-9B94-346929B83360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF2C67C2-7C58-4A0B-BB3E-E54DFE0219D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -134,15 +134,6 @@
     <t>mean_MAD</t>
   </si>
   <si>
-    <t>Precision (inter batch)</t>
-  </si>
-  <si>
-    <t>Precision (intra batch)</t>
-  </si>
-  <si>
-    <t>Linearity</t>
-  </si>
-  <si>
     <t>Coefficient of variation of technical replicates (%CV)</t>
   </si>
   <si>
@@ -152,40 +143,49 @@
     <t>Linearity of response of varying ratios of blood (high mutation) and sperm (low mutation) from the same donor (R^2)</t>
   </si>
   <si>
-    <t>External concodance (blood)</t>
-  </si>
-  <si>
-    <t>External concordance (sperm)</t>
-  </si>
-  <si>
     <t>NA</t>
   </si>
   <si>
     <t>Number of SNVs per diploid genome is similar to past studies (mean)</t>
   </si>
   <si>
-    <t>Robustness</t>
-  </si>
-  <si>
     <t>Percentage of samples that meet all non-negotiable metrics (including samples which failed processing)</t>
   </si>
   <si>
-    <t>Uniformity (SNV position)</t>
-  </si>
-  <si>
-    <t>Uniformity (SNV spacing)</t>
-  </si>
-  <si>
-    <t>Uniformity (chromosomal SNV rate)</t>
-  </si>
-  <si>
-    <t>Cross-reactivity (recurrent variants)</t>
-  </si>
-  <si>
-    <t>External concordance (trinucleotide context)</t>
-  </si>
-  <si>
-    <t>Cross-reactivity (germline contamination)</t>
+    <t>uniformity_SNV_position</t>
+  </si>
+  <si>
+    <t>uniformity_SNV_spacing</t>
+  </si>
+  <si>
+    <t>uniformity_chromosomal_SNV_rate</t>
+  </si>
+  <si>
+    <t>cross_reactivity _recurrent_variants</t>
+  </si>
+  <si>
+    <t>cross_reactivity_germline_contamination</t>
+  </si>
+  <si>
+    <t>external_concordance_trinuc_context</t>
+  </si>
+  <si>
+    <t>external_concordance_sperm</t>
+  </si>
+  <si>
+    <t>external concodance_blood</t>
+  </si>
+  <si>
+    <t>precision_intra_batch</t>
+  </si>
+  <si>
+    <t>precision_inter_batch</t>
+  </si>
+  <si>
+    <t>linearity</t>
+  </si>
+  <si>
+    <t>robustness</t>
   </si>
 </sst>
 </file>
@@ -1112,7 +1112,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
         <v>30</v>
@@ -1147,7 +1147,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B3" t="s">
         <v>26</v>
@@ -1182,7 +1182,7 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
@@ -1217,7 +1217,7 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B5" t="s">
         <v>17</v>
@@ -1252,7 +1252,7 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
         <v>21</v>
@@ -1287,7 +1287,7 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
         <v>13</v>
@@ -1322,16 +1322,16 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
         <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -1349,24 +1349,24 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="K8" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E9">
         <v>500</v>
@@ -1384,24 +1384,24 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="K9" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" t="s">
         <v>32</v>
-      </c>
-      <c r="B10" t="s">
-        <v>35</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -1419,24 +1419,24 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="K10" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" t="s">
         <v>33</v>
-      </c>
-      <c r="B11" t="s">
-        <v>36</v>
       </c>
       <c r="C11" t="s">
         <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E11">
         <v>0.9</v>
@@ -1454,24 +1454,24 @@
         <v>0</v>
       </c>
       <c r="J11" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="K11" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" t="s">
         <v>34</v>
-      </c>
-      <c r="B12" t="s">
-        <v>37</v>
       </c>
       <c r="C12" t="s">
         <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E12">
         <v>0.9</v>
@@ -1489,24 +1489,24 @@
         <v>0</v>
       </c>
       <c r="J12" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="K12" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="B13" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C13" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D13" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E13">
         <v>90</v>
@@ -1524,10 +1524,10 @@
         <v>0</v>
       </c>
       <c r="J13" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="K13" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
1. Renamed reccurant variatns metric 2. Updated to use percentage rather thn absolute value 3. updated thresholds
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF2C67C2-7C58-4A0B-BB3E-E54DFE0219D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1097B99-F06D-4E93-BD32-72634F513AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -89,15 +89,9 @@
     <t>gini_coefficient</t>
   </si>
   <si>
-    <t>Number of somatic variant calls that occur more than once in a batch, without a plausible biological explanation</t>
-  </si>
-  <si>
     <t>Batch</t>
   </si>
   <si>
-    <t>total_recurrent_variants</t>
-  </si>
-  <si>
     <t>_recurrent_variant_metrics.json</t>
   </si>
   <si>
@@ -161,9 +155,6 @@
     <t>uniformity_chromosomal_SNV_rate</t>
   </si>
   <si>
-    <t>cross_reactivity _recurrent_variants</t>
-  </si>
-  <si>
     <t>cross_reactivity_germline_contamination</t>
   </si>
   <si>
@@ -186,6 +177,15 @@
   </si>
   <si>
     <t>robustness</t>
+  </si>
+  <si>
+    <t>cross_reactivity_inter_sample_reccurance</t>
+  </si>
+  <si>
+    <t>pct_recurrent_variants</t>
+  </si>
+  <si>
+    <t>Percentage of variants that are called in more than one sample</t>
   </si>
 </sst>
 </file>
@@ -675,9 +675,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1112,10 +1113,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -1139,18 +1140,18 @@
         <v>1</v>
       </c>
       <c r="J2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K2" t="s">
         <v>29</v>
-      </c>
-      <c r="K2" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
@@ -1174,15 +1175,15 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="K3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
@@ -1215,47 +1216,47 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B5" t="s">
+    <row r="5" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="E5" s="2">
+        <v>0</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0</v>
+      </c>
+      <c r="I5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-      <c r="I5" t="b">
-        <v>1</v>
-      </c>
-      <c r="J5" t="s">
-        <v>20</v>
-      </c>
-      <c r="K5" t="s">
-        <v>19</v>
+      <c r="K5" s="2" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C6" t="s">
         <v>12</v>
@@ -1279,15 +1280,15 @@
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s">
         <v>13</v>
@@ -1314,24 +1315,24 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="K7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C8" t="s">
         <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -1349,24 +1350,24 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E9">
         <v>500</v>
@@ -1384,24 +1385,24 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -1419,24 +1420,24 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
         <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E11">
         <v>0.9</v>
@@ -1454,24 +1455,24 @@
         <v>0</v>
       </c>
       <c r="J11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B12" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C12" t="s">
         <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E12">
         <v>0.9</v>
@@ -1489,24 +1490,24 @@
         <v>0</v>
       </c>
       <c r="J12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E13">
         <v>90</v>
@@ -1524,10 +1525,10 @@
         <v>0</v>
       </c>
       <c r="J13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Integrated new script into pipeline
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1097B99-F06D-4E93-BD32-72634F513AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F126CE3B-2F96-4421-8DB4-99A97A1B4BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -179,13 +179,13 @@
     <t>robustness</t>
   </si>
   <si>
-    <t>cross_reactivity_inter_sample_reccurance</t>
-  </si>
-  <si>
-    <t>pct_recurrent_variants</t>
-  </si>
-  <si>
     <t>Percentage of variants that are called in more than one sample</t>
+  </si>
+  <si>
+    <t>cross_reactivity_recurrant_variants</t>
+  </si>
+  <si>
+    <t>percentage_recurrent_variants.value</t>
   </si>
 </sst>
 </file>
@@ -675,10 +675,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1066,7 +1065,7 @@
   <dimension ref="A1:K13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="41.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.90625" customWidth="1"/>
     <col min="2" max="2" width="101.7265625" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="35.26953125" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
@@ -1216,39 +1215,39 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0.5</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K5" t="s">
         <v>49</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" s="2">
-        <v>0</v>
-      </c>
-      <c r="F5" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="G5" s="2">
-        <v>0</v>
-      </c>
-      <c r="H5" s="2">
-        <v>0</v>
-      </c>
-      <c r="I5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Updated nn threshold for external_concordance_trinuc_context
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39746353-06F5-40C7-A88B-5D7DFBB51C70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E012E2B0-782D-4DC6-B3E2-54F26A0AA602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -1303,7 +1303,7 @@
         <v>11</v>
       </c>
       <c r="E7">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="F7">
         <v>1</v>

</xml_diff>

<commit_message>
Finished adding germline_overlap metric, all tests passing
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1CD2039-9FBD-4A5B-AEF9-1347DEC58D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{878B4D80-AAAE-4F4C-A0DB-0115AC27B1F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -86,15 +86,6 @@
     <t>_recurrent_variant_metrics.json</t>
   </si>
   <si>
-    <t>Percentage of somatic variants that are germline contaminants</t>
-  </si>
-  <si>
-    <t>percent_germline_contamination</t>
-  </si>
-  <si>
-    <t>_germline_contamination_metrics.json</t>
-  </si>
-  <si>
     <t>_trinuc_similarities.csv</t>
   </si>
   <si>
@@ -131,9 +122,6 @@
     <t>uniformity_SNV_spacing</t>
   </si>
   <si>
-    <t>cross_reactivity_germline_contamination</t>
-  </si>
-  <si>
     <t>external_concordance_trinuc_context</t>
   </si>
   <si>
@@ -171,6 +159,18 @@
   </si>
   <si>
     <t>external_concordance_blood</t>
+  </si>
+  <si>
+    <t>cross_reactivity_gnomAD_overlap</t>
+  </si>
+  <si>
+    <t>Rate of SNVs that overlap with gnomAD per evaluated base</t>
+  </si>
+  <si>
+    <t>_gnomAD_overlap_metrics.json</t>
+  </si>
+  <si>
+    <t>rate_gnomAD_overlap.value</t>
   </si>
 </sst>
 </file>
@@ -1098,10 +1098,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -1125,18 +1125,18 @@
         <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="K2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
@@ -1160,18 +1160,18 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="K3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
         <v>12</v>
@@ -1198,15 +1198,15 @@
         <v>15</v>
       </c>
       <c r="K4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
@@ -1218,27 +1218,27 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I5" t="b">
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="K5" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
         <v>13</v>
@@ -1265,24 +1265,24 @@
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="K6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E7" s="2">
         <v>5.0000000000000001E-9</v>
@@ -1300,24 +1300,24 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="K7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
         <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E8" s="2">
         <v>7.4999999999999997E-8</v>
@@ -1335,24 +1335,24 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="K8" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -1370,24 +1370,24 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="K9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E10">
         <v>0.9</v>
@@ -1405,24 +1405,24 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="K10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C11" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E11">
         <v>90</v>
@@ -1440,10 +1440,10 @@
         <v>0</v>
       </c>
       <c r="J11" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="K11" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Set targets for gnomAD overlap
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{878B4D80-AAAE-4F4C-A0DB-0115AC27B1F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{099A8722-E6C7-40A4-8D10-286EBA8E522A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -1217,14 +1217,14 @@
       <c r="E5">
         <v>0</v>
       </c>
-      <c r="F5">
-        <v>0</v>
+      <c r="F5" s="2">
+        <v>2.51E-8</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
-      <c r="H5">
-        <v>0</v>
+      <c r="H5" s="2">
+        <v>1.0039999999999999E-8</v>
       </c>
       <c r="I5" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Revert "Merge pull request #222 from systematicmedicine/feature/germline-overlap-rate"
This reverts commit 53db7710e0b92fc714e3ed3ea99acb5ae72b53b7, reversing
changes made to cec803fae66580ff448cd2fca5c6bff35f1684c2.
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{099A8722-E6C7-40A4-8D10-286EBA8E522A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1CD2039-9FBD-4A5B-AEF9-1347DEC58D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -86,6 +86,15 @@
     <t>_recurrent_variant_metrics.json</t>
   </si>
   <si>
+    <t>Percentage of somatic variants that are germline contaminants</t>
+  </si>
+  <si>
+    <t>percent_germline_contamination</t>
+  </si>
+  <si>
+    <t>_germline_contamination_metrics.json</t>
+  </si>
+  <si>
     <t>_trinuc_similarities.csv</t>
   </si>
   <si>
@@ -122,6 +131,9 @@
     <t>uniformity_SNV_spacing</t>
   </si>
   <si>
+    <t>cross_reactivity_germline_contamination</t>
+  </si>
+  <si>
     <t>external_concordance_trinuc_context</t>
   </si>
   <si>
@@ -159,18 +171,6 @@
   </si>
   <si>
     <t>external_concordance_blood</t>
-  </si>
-  <si>
-    <t>cross_reactivity_gnomAD_overlap</t>
-  </si>
-  <si>
-    <t>Rate of SNVs that overlap with gnomAD per evaluated base</t>
-  </si>
-  <si>
-    <t>_gnomAD_overlap_metrics.json</t>
-  </si>
-  <si>
-    <t>rate_gnomAD_overlap.value</t>
   </si>
 </sst>
 </file>
@@ -1098,10 +1098,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -1125,18 +1125,18 @@
         <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="K2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
@@ -1160,18 +1160,18 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="K3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
         <v>12</v>
@@ -1198,15 +1198,15 @@
         <v>15</v>
       </c>
       <c r="K4" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="B5" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
@@ -1217,28 +1217,28 @@
       <c r="E5">
         <v>0</v>
       </c>
-      <c r="F5" s="2">
-        <v>2.51E-8</v>
+      <c r="F5">
+        <v>5</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
-      <c r="H5" s="2">
-        <v>1.0039999999999999E-8</v>
+      <c r="H5">
+        <v>2</v>
       </c>
       <c r="I5" t="b">
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="K5" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s">
         <v>13</v>
@@ -1265,24 +1265,24 @@
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="K6" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E7" s="2">
         <v>5.0000000000000001E-9</v>
@@ -1300,24 +1300,24 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="K7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" t="s">
         <v>40</v>
-      </c>
-      <c r="B8" t="s">
-        <v>36</v>
       </c>
       <c r="C8" t="s">
         <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E8" s="2">
         <v>7.4999999999999997E-8</v>
@@ -1335,24 +1335,24 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="K8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -1370,24 +1370,24 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="K9" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E10">
         <v>0.9</v>
@@ -1405,24 +1405,24 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="K10" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E11">
         <v>90</v>
@@ -1440,10 +1440,10 @@
         <v>0</v>
       </c>
       <c r="J11" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="K11" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cross_reactivity_gnomAD_overlap reverted to drawing from percent_gnomAD_overlap rather than rate_gnomAD_overlap
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21CB7C8D-CB77-4486-B1CB-D2F773982330}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91C0EBFA-CE67-4433-88FE-853DC03B624B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -164,9 +164,6 @@
     <t>_gnomAD_overlap_metrics.json</t>
   </si>
   <si>
-    <t>rate_gnomAD_overlap.value</t>
-  </si>
-  <si>
     <t>precision_inter_batch</t>
   </si>
   <si>
@@ -189,6 +186,9 @@
   </si>
   <si>
     <t>snv_rate.value</t>
+  </si>
+  <si>
+    <t>percent_gnomAD_overlap.value</t>
   </si>
 </sst>
 </file>
@@ -1236,13 +1236,13 @@
         <v>0</v>
       </c>
       <c r="F5" s="2">
-        <v>2.51E-8</v>
+        <v>5</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5" s="2">
-        <v>1.0039999999999999E-8</v>
+        <v>2</v>
       </c>
       <c r="I5" t="b">
         <v>1</v>
@@ -1251,7 +1251,7 @@
         <v>41</v>
       </c>
       <c r="K5" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
@@ -1318,10 +1318,10 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
+        <v>48</v>
+      </c>
+      <c r="K7" t="s">
         <v>49</v>
-      </c>
-      <c r="K7" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
@@ -1353,18 +1353,18 @@
         <v>1</v>
       </c>
       <c r="J8" t="s">
+        <v>48</v>
+      </c>
+      <c r="K8" t="s">
         <v>49</v>
-      </c>
-      <c r="K8" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" t="s">
         <v>44</v>
-      </c>
-      <c r="B9" t="s">
-        <v>45</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
@@ -1396,10 +1396,10 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
@@ -1431,10 +1431,10 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C11" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
Precision now used normalised IQR instead of coefficient of variation (change to mon parametric measure of precision)
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91C0EBFA-CE67-4433-88FE-853DC03B624B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B14576E-E546-467E-8973-BB3CC8500EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -170,9 +170,6 @@
     <t>precision_intra_batch_snv</t>
   </si>
   <si>
-    <t>Coefficient of variation of SNV rate, for technical replicates (%CV)</t>
-  </si>
-  <si>
     <t>TBD measure of inter batch variation</t>
   </si>
   <si>
@@ -189,6 +186,9 @@
   </si>
   <si>
     <t>percent_gnomAD_overlap.value</t>
+  </si>
+  <si>
+    <t>Normalised IQR of SNV rate, for technical replicates (%normIQR)</t>
   </si>
 </sst>
 </file>
@@ -1251,7 +1251,7 @@
         <v>41</v>
       </c>
       <c r="K5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
@@ -1318,10 +1318,10 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
+        <v>47</v>
+      </c>
+      <c r="K7" t="s">
         <v>48</v>
-      </c>
-      <c r="K7" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
@@ -1353,10 +1353,10 @@
         <v>1</v>
       </c>
       <c r="J8" t="s">
+        <v>47</v>
+      </c>
+      <c r="K8" t="s">
         <v>48</v>
-      </c>
-      <c r="K8" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
@@ -1364,7 +1364,7 @@
         <v>43</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
@@ -1396,10 +1396,10 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
@@ -1434,7 +1434,7 @@
         <v>42</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C11" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
Increased non-negotiable upper threshold for cross_reactivity_gnomAD_overlap system metric from 5 to 10
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\SomaticCODEC\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B14576E-E546-467E-8973-BB3CC8500EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E64C212-2B95-41D5-94AC-020FB2C8A08A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -1067,19 +1067,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
   <dimension ref="A1:K13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.81640625" customWidth="1"/>
-    <col min="2" max="2" width="122.453125" customWidth="1"/>
-    <col min="3" max="4" width="35.26953125" customWidth="1"/>
+    <col min="1" max="1" width="35.85546875" customWidth="1"/>
+    <col min="2" max="2" width="122.42578125" customWidth="1"/>
+    <col min="3" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.81640625" customWidth="1"/>
-    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="54" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -1114,7 +1114,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -1149,7 +1149,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -1184,7 +1184,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -1219,7 +1219,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>39</v>
       </c>
@@ -1236,7 +1236,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="2">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -1254,7 +1254,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -1289,7 +1289,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -1324,7 +1324,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>38</v>
       </c>
@@ -1359,7 +1359,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>43</v>
       </c>
@@ -1394,7 +1394,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>46</v>
       </c>
@@ -1429,7 +1429,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>42</v>
       </c>
@@ -1464,7 +1464,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -1499,7 +1499,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>30</v>
       </c>

</xml_diff>

<commit_message>
uniformity_SNV_spacing system metric now uses 10th percentile, ideal thresholds updated based on buffy coat data
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E64C212-2B95-41D5-94AC-020FB2C8A08A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A094827E-3592-416A-BB77-9A37D5929F55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -92,15 +92,9 @@
     <t>^Abascal-2021-granulocyte,(?P&lt;val&gt;[0-9.]+)$</t>
   </si>
   <si>
-    <t>5th percentile of distance of each SNV to nearest SNV</t>
-  </si>
-  <si>
     <t>_snv_distance.json</t>
   </si>
   <si>
-    <t>percentiles.5</t>
-  </si>
-  <si>
     <t>_snv_position_metrics.json</t>
   </si>
   <si>
@@ -189,6 +183,12 @@
   </si>
   <si>
     <t>Normalised IQR of SNV rate, for technical replicates (%normIQR)</t>
+  </si>
+  <si>
+    <t>percentiles.10</t>
+  </si>
+  <si>
+    <t>10th percentile of distance of each SNV to nearest SNV</t>
   </si>
 </sst>
 </file>
@@ -1116,10 +1116,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -1143,18 +1143,18 @@
         <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
@@ -1169,27 +1169,27 @@
         <v>3000000</v>
       </c>
       <c r="G3">
-        <v>1000</v>
+        <v>44495</v>
       </c>
       <c r="H3">
-        <v>1500000</v>
+        <v>263304</v>
       </c>
       <c r="I3" t="b">
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K3" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
         <v>12</v>
@@ -1216,15 +1216,15 @@
         <v>15</v>
       </c>
       <c r="K4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
@@ -1248,15 +1248,15 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="K5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B6" t="s">
         <v>13</v>
@@ -1291,16 +1291,16 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E7" s="2">
         <v>5.0000000000000001E-9</v>
@@ -1318,24 +1318,24 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="K7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
         <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E8" s="2">
         <v>7.4999999999999997E-8</v>
@@ -1353,24 +1353,24 @@
         <v>1</v>
       </c>
       <c r="J8" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="K8" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -1388,94 +1388,94 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I10" t="b">
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" t="s">
         <v>42</v>
-      </c>
-      <c r="B11" t="s">
-        <v>44</v>
       </c>
       <c r="C11" t="s">
         <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I11" t="b">
         <v>0</v>
       </c>
       <c r="J11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C12" t="s">
         <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E12">
         <v>0.9</v>
@@ -1493,24 +1493,24 @@
         <v>0</v>
       </c>
       <c r="J12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E13">
         <v>90</v>
@@ -1528,10 +1528,10 @@
         <v>0</v>
       </c>
       <c r="J13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Icreased uniformity_SNV_spacing nn lower from 100 to 120
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A094827E-3592-416A-BB77-9A37D5929F55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90EBB5F7-062B-4984-96FF-ACF4438ED969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -1163,7 +1163,7 @@
         <v>11</v>
       </c>
       <c r="E3">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="F3">
         <v>3000000</v>

</xml_diff>

<commit_message>
Increased non-negotiable upper threshold for uniformity_SNV_position system metric from 15 to 20.1
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90EBB5F7-062B-4984-96FF-ACF4438ED969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8980B87B-C2BA-4147-8FCE-CD1B5186CD3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -1131,7 +1131,7 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>15</v>
+        <v>20.100000000000001</v>
       </c>
       <c r="G2">
         <v>0</v>

</xml_diff>

<commit_message>
Updated non-negotiable upper threshold for uniformity_SNV_position
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8980B87B-C2BA-4147-8FCE-CD1B5186CD3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{127471E7-3550-4598-B773-3171BF37E5D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -1131,7 +1131,7 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>20.100000000000001</v>
+        <v>15.5</v>
       </c>
       <c r="G2">
         <v>0</v>

</xml_diff>

<commit_message>
Updated nn thresholds for uniformity_SNV_position and uniformity_SNV_spacing
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{127471E7-3550-4598-B773-3171BF37E5D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92AB6EC7-5C08-4180-9A05-E5F1A63565C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -185,10 +185,10 @@
     <t>Normalised IQR of SNV rate, for technical replicates (%normIQR)</t>
   </si>
   <si>
-    <t>percentiles.10</t>
-  </si>
-  <si>
-    <t>10th percentile of distance of each SNV to nearest SNV</t>
+    <t>5th percentile of distance of each SNV to nearest SNV</t>
+  </si>
+  <si>
+    <t>percentiles.5</t>
   </si>
 </sst>
 </file>
@@ -1131,7 +1131,7 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>15.5</v>
+        <v>20</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -1154,7 +1154,7 @@
         <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
@@ -1169,10 +1169,10 @@
         <v>3000000</v>
       </c>
       <c r="G3">
-        <v>44495</v>
+        <v>1000</v>
       </c>
       <c r="H3">
-        <v>263304</v>
+        <v>1500000</v>
       </c>
       <c r="I3" t="b">
         <v>1</v>
@@ -1181,7 +1181,7 @@
         <v>18</v>
       </c>
       <c r="K3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Removed inter-batch precision system metric
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92AB6EC7-5C08-4180-9A05-E5F1A63565C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21D80068-3495-4108-847C-5467EC2FD0AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$82</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="49">
   <si>
     <t>nn_lower</t>
   </si>
@@ -158,13 +158,7 @@
     <t>_gnomAD_overlap_metrics.json</t>
   </si>
   <si>
-    <t>precision_inter_batch</t>
-  </si>
-  <si>
     <t>precision_intra_batch_snv</t>
-  </si>
-  <si>
-    <t>TBD measure of inter batch variation</t>
   </si>
   <si>
     <t>TBD measure of trinucleotide convtext precision, within technical replicates</t>
@@ -1066,7 +1060,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.85546875" customWidth="1"/>
@@ -1154,7 +1148,7 @@
         <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
@@ -1181,7 +1175,7 @@
         <v>18</v>
       </c>
       <c r="K3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -1251,7 +1245,7 @@
         <v>39</v>
       </c>
       <c r="K5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -1318,10 +1312,10 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -1353,18 +1347,18 @@
         <v>1</v>
       </c>
       <c r="J8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K8" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
@@ -1396,10 +1390,10 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
@@ -1431,10 +1425,10 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s">
         <v>12</v>
@@ -1442,17 +1436,17 @@
       <c r="D11" t="s">
         <v>21</v>
       </c>
-      <c r="E11" t="s">
-        <v>21</v>
-      </c>
-      <c r="F11" t="s">
-        <v>21</v>
-      </c>
-      <c r="G11" t="s">
-        <v>21</v>
-      </c>
-      <c r="H11" t="s">
-        <v>21</v>
+      <c r="E11">
+        <v>0.9</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>0.95</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
       </c>
       <c r="I11" t="b">
         <v>0</v>
@@ -1466,28 +1460,28 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="D12" t="s">
         <v>21</v>
       </c>
       <c r="E12">
-        <v>0.9</v>
+        <v>90</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="G12">
-        <v>0.95</v>
+        <v>95</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I12" t="b">
         <v>0</v>
@@ -1499,43 +1493,8 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" t="s">
-        <v>22</v>
-      </c>
-      <c r="C13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" t="s">
-        <v>21</v>
-      </c>
-      <c r="E13">
-        <v>90</v>
-      </c>
-      <c r="F13">
-        <v>100</v>
-      </c>
-      <c r="G13">
-        <v>95</v>
-      </c>
-      <c r="H13">
-        <v>100</v>
-      </c>
-      <c r="I13" t="b">
-        <v>0</v>
-      </c>
-      <c r="J13" t="s">
-        <v>21</v>
-      </c>
-      <c r="K13" t="s">
-        <v>21</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K83" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K82" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated regex for external_concordance_trinuc_context in system_level_metrics.xlsx
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21D80068-3495-4108-847C-5467EC2FD0AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF1A3F6C-01C8-4D5C-859D-BA83E2D8BB51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -77,9 +77,6 @@
     <t>EX call somatic variants</t>
   </si>
   <si>
-    <t>Cosine similarity score for trinucleotide context compared with established signatures from past studies</t>
-  </si>
-  <si>
     <t>Batch</t>
   </si>
   <si>
@@ -89,9 +86,6 @@
     <t>_trinuc_similarities.csv</t>
   </si>
   <si>
-    <t>^Abascal-2021-granulocyte,(?P&lt;val&gt;[0-9.]+)$</t>
-  </si>
-  <si>
     <t>_snv_distance.json</t>
   </si>
   <si>
@@ -183,6 +177,12 @@
   </si>
   <si>
     <t>percentiles.5</t>
+  </si>
+  <si>
+    <t>^Abascal-2021-granulocyte,[^,]+,(?P&lt;val&gt;[0-9.]+)$</t>
+  </si>
+  <si>
+    <t>Cosine similarity score for normalised trinucleotide context compared with established signatures from past studies</t>
   </si>
 </sst>
 </file>
@@ -1110,10 +1110,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -1137,18 +1137,18 @@
         <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="K2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
@@ -1172,24 +1172,24 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="K3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1207,18 +1207,18 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
@@ -1242,18 +1242,18 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="K5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="C6" t="s">
         <v>12</v>
@@ -1277,24 +1277,24 @@
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K6" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E7" s="2">
         <v>5.0000000000000001E-9</v>
@@ -1312,24 +1312,24 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="K7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C8" t="s">
         <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E8" s="2">
         <v>7.4999999999999997E-8</v>
@@ -1347,24 +1347,24 @@
         <v>1</v>
       </c>
       <c r="J8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="K8" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -1382,59 +1382,59 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E10" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F10" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G10" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H10" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I10" t="b">
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K10" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C11" t="s">
         <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E11">
         <v>0.9</v>
@@ -1452,24 +1452,24 @@
         <v>0</v>
       </c>
       <c r="J11" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K11" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C12" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D12" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E12">
         <v>90</v>
@@ -1487,10 +1487,10 @@
         <v>0</v>
       </c>
       <c r="J12" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K12" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed nn thresholds for external_concordance_blood, removed ideal thresholds
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\SomaticCODEC\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8656C732-F374-4233-9B14-27ABBE838A0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F5D1FF-E908-49B7-BC0B-83ACFFF0ECA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -1061,19 +1061,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
   <dimension ref="A1:K12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.81640625" customWidth="1"/>
-    <col min="2" max="2" width="122.453125" customWidth="1"/>
-    <col min="3" max="4" width="35.26953125" customWidth="1"/>
+    <col min="1" max="1" width="35.85546875" customWidth="1"/>
+    <col min="2" max="2" width="122.42578125" customWidth="1"/>
+    <col min="3" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.81640625" customWidth="1"/>
-    <col min="10" max="10" width="40.36328125" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="40.42578125" customWidth="1"/>
     <col min="11" max="11" width="54" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -1108,7 +1108,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -1143,7 +1143,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -1178,7 +1178,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -1213,7 +1213,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -1248,7 +1248,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -1318,7 +1318,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -1332,17 +1332,13 @@
         <v>15</v>
       </c>
       <c r="E8" s="2">
-        <v>7.4999999999999997E-8</v>
+        <v>2.22E-7</v>
       </c>
       <c r="F8" s="2">
-        <v>5.0200000000000002E-7</v>
-      </c>
-      <c r="G8" s="2">
-        <v>1.35E-7</v>
-      </c>
-      <c r="H8" s="2">
-        <v>3.6800000000000001E-7</v>
-      </c>
+        <v>6.1399999999999997E-7</v>
+      </c>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
       <c r="I8" t="b">
         <v>1</v>
       </c>
@@ -1353,7 +1349,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>33</v>
       </c>
@@ -1388,7 +1384,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>35</v>
       </c>
@@ -1423,7 +1419,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -1458,7 +1454,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>22</v>
       </c>

</xml_diff>

<commit_message>
Updated ex_snv_read_position_metrics.py and test, added system metric
</commit_message>
<xml_diff>
--- a/config/system_level_metrics.xlsx
+++ b/config/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93D6CF3-4F8A-4148-87A7-15A80A2E87EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{381716B7-1C21-469E-994C-E6D7063F4DC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$83</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="53">
   <si>
     <t>nn_lower</t>
   </si>
@@ -183,6 +183,18 @@
   </si>
   <si>
     <t>Linearity of response to different ratios of blood (high mutation) and sperm (low mutation) from the same donor (R^2)</t>
+  </si>
+  <si>
+    <t>uniformity_SNV_read_position</t>
+  </si>
+  <si>
+    <t>Maximum absolute difference between empirical and uniform cumulative distribution functions for SNV read positions</t>
+  </si>
+  <si>
+    <t>cdf_max_difference.value</t>
+  </si>
+  <si>
+    <t>EX.MET_SNV_READ_POSITION_JSON</t>
   </si>
 </sst>
 </file>
@@ -672,11 +684,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1061,7 +1072,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.85546875" customWidth="1"/>
@@ -1182,80 +1193,80 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="C4" t="s">
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>0.5</v>
+        <v>0.05</v>
       </c>
       <c r="G4">
         <v>0</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I4" t="b">
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="K4" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
-      <c r="F5" s="3">
-        <v>10</v>
+      <c r="F5">
+        <v>0.5</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
-      <c r="H5" s="3">
-        <v>2</v>
+      <c r="H5">
+        <v>0</v>
       </c>
       <c r="I5" t="b">
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="K5" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
         <v>12</v>
@@ -1264,68 +1275,68 @@
         <v>11</v>
       </c>
       <c r="E6">
-        <v>0.85</v>
+        <v>0</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G6">
-        <v>0.95</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I6" t="b">
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="2">
-        <v>5.0000000000000001E-9</v>
-      </c>
-      <c r="F7" s="2">
-        <v>4.9999999999999998E-8</v>
-      </c>
-      <c r="G7" s="2">
-        <v>8.9999999999999995E-9</v>
-      </c>
-      <c r="H7" s="2">
-        <v>3.7E-8</v>
+        <v>11</v>
+      </c>
+      <c r="E7">
+        <v>0.85</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>0.95</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
       </c>
       <c r="I7" t="b">
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="K7" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C8" t="s">
         <v>12</v>
@@ -1334,13 +1345,17 @@
         <v>14</v>
       </c>
       <c r="E8" s="2">
-        <v>2.22E-7</v>
+        <v>5.0000000000000001E-9</v>
       </c>
       <c r="F8" s="2">
-        <v>6.1399999999999997E-7</v>
-      </c>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
+        <v>4.9999999999999998E-8</v>
+      </c>
+      <c r="G8" s="2">
+        <v>8.9999999999999995E-9</v>
+      </c>
+      <c r="H8" s="2">
+        <v>3.7E-8</v>
+      </c>
       <c r="I8" t="b">
         <v>1</v>
       </c>
@@ -1353,10 +1368,10 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
@@ -1364,34 +1379,30 @@
       <c r="D9" t="s">
         <v>14</v>
       </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9">
-        <v>20</v>
-      </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
-      <c r="H9">
-        <v>10</v>
-      </c>
+      <c r="E9" s="2">
+        <v>2.22E-7</v>
+      </c>
+      <c r="F9" s="2">
+        <v>6.1399999999999997E-7</v>
+      </c>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
       <c r="I9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="K9" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
@@ -1399,17 +1410,17 @@
       <c r="D10" t="s">
         <v>14</v>
       </c>
-      <c r="E10" t="s">
-        <v>14</v>
-      </c>
-      <c r="F10" t="s">
-        <v>14</v>
-      </c>
-      <c r="G10" t="s">
-        <v>14</v>
-      </c>
-      <c r="H10" t="s">
-        <v>14</v>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>20</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>10</v>
       </c>
       <c r="I10" t="b">
         <v>0</v>
@@ -1423,10 +1434,10 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C11" t="s">
         <v>12</v>
@@ -1434,17 +1445,17 @@
       <c r="D11" t="s">
         <v>14</v>
       </c>
-      <c r="E11">
-        <v>0.9</v>
-      </c>
-      <c r="F11">
-        <v>1</v>
-      </c>
-      <c r="G11">
-        <v>0.95</v>
-      </c>
-      <c r="H11">
-        <v>1</v>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H11" t="s">
+        <v>14</v>
       </c>
       <c r="I11" t="b">
         <v>0</v>
@@ -1458,28 +1469,28 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="C12" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D12" t="s">
         <v>14</v>
       </c>
       <c r="E12">
-        <v>90</v>
+        <v>0.9</v>
       </c>
       <c r="F12">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G12">
-        <v>95</v>
+        <v>0.95</v>
       </c>
       <c r="H12">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="I12" t="b">
         <v>0</v>
@@ -1491,8 +1502,43 @@
         <v>14</v>
       </c>
     </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13">
+        <v>90</v>
+      </c>
+      <c r="F13">
+        <v>100</v>
+      </c>
+      <c r="G13">
+        <v>95</v>
+      </c>
+      <c r="H13">
+        <v>100</v>
+      </c>
+      <c r="I13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J13" t="s">
+        <v>14</v>
+      </c>
+      <c r="K13" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K82" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K83" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>